<commit_message>
Updated NOR_grids_kan50 model - 2026-09-22 15:26
</commit_message>
<xml_diff>
--- a/VerveStacks_NOR_grids_kan50/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_NOR_grids_kan50/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_NOR_grids_kan50\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B230EF5E-2E7F-40EE-AA22-1CDB92AEE68F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0DFA6E35-B205-4DF0-80CF-8B376E3067E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4012" yWindow="4012" windowWidth="21601" windowHeight="11423" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3331,7 +3331,7 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AF7DB727-4801-4965-AF81-F5B9A31D77BF}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6DF6544C-C0A4-4F9F-9B9C-8E090AEBC833}">
   <dimension ref="B9:L122"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -30661,7 +30661,7 @@
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6C7552EF-B29A-431B-B1D2-EF5F633621EE}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6D184941-B119-4257-9E15-5DFAA4E5AD34}">
   <dimension ref="B9:H122"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>